<commit_message>
Added asia results for dlama and fixed size of a few graph. llama 3b needs to be tested next
</commit_message>
<xml_diff>
--- a/correlation_analysis/benchmark_correlation_Llama_3_2-3B.xlsx
+++ b/correlation_analysis/benchmark_correlation_Llama_3_2-3B.xlsx
@@ -442,7 +442,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>DLAMA</t>
+          <t>GeoMLAMA</t>
         </is>
       </c>
     </row>
@@ -456,10 +456,10 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>0.8986776749886862</v>
+        <v>0.4131006675953109</v>
       </c>
       <c r="D2" t="n">
-        <v>0.3500111183545106</v>
+        <v>0.31012627315061</v>
       </c>
     </row>
     <row r="3">
@@ -469,26 +469,26 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.8986776749886862</v>
+        <v>0.4131006675953109</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>0.180961116582101</v>
+        <v>-0.2606795377402163</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>DLAMA</t>
+          <t>GeoMLAMA</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.3500111183545106</v>
+        <v>0.31012627315061</v>
       </c>
       <c r="C4" t="n">
-        <v>0.180961116582101</v>
+        <v>-0.2606795377402163</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
@@ -521,7 +521,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>DLAMA</t>
+          <t>GeoMLAMA</t>
         </is>
       </c>
     </row>
@@ -535,10 +535,10 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>0.01487922200579105</v>
+        <v>0.5868993324046889</v>
       </c>
       <c r="D2" t="n">
-        <v>0.4964228655307756</v>
+        <v>0.68987372684939</v>
       </c>
     </row>
     <row r="3">
@@ -548,26 +548,26 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.01487922200579105</v>
+        <v>0.5868993324046889</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>0.7315212852478248</v>
+        <v>0.7393204622597835</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>DLAMA</t>
+          <t>GeoMLAMA</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.4964228655307756</v>
+        <v>0.68987372684939</v>
       </c>
       <c r="C4" t="n">
-        <v>0.7315212852478248</v>
+        <v>0.7393204622597835</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
updated dlama finalized results
</commit_message>
<xml_diff>
--- a/correlation_analysis/benchmark_correlation_Llama_3_2-3B.xlsx
+++ b/correlation_analysis/benchmark_correlation_Llama_3_2-3B.xlsx
@@ -442,7 +442,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>GeoMLAMA</t>
+          <t>DLAMA</t>
         </is>
       </c>
     </row>
@@ -456,10 +456,10 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>0.4131006675953109</v>
+        <v>0.8986776749886862</v>
       </c>
       <c r="D2" t="n">
-        <v>0.31012627315061</v>
+        <v>0.1659741993200967</v>
       </c>
     </row>
     <row r="3">
@@ -469,26 +469,26 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.4131006675953109</v>
+        <v>0.8986776749886862</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.2606795377402163</v>
+        <v>-0.162224249290581</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>GeoMLAMA</t>
+          <t>DLAMA</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.31012627315061</v>
+        <v>0.1659741993200967</v>
       </c>
       <c r="C4" t="n">
-        <v>-0.2606795377402163</v>
+        <v>-0.162224249290581</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
@@ -521,7 +521,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>GeoMLAMA</t>
+          <t>DLAMA</t>
         </is>
       </c>
     </row>
@@ -535,10 +535,10 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>0.5868993324046889</v>
+        <v>0.01487922200579105</v>
       </c>
       <c r="D2" t="n">
-        <v>0.68987372684939</v>
+        <v>0.7533247827402964</v>
       </c>
     </row>
     <row r="3">
@@ -548,26 +548,26 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.5868993324046889</v>
+        <v>0.01487922200579105</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>0.7393204622597835</v>
+        <v>0.7587982300872619</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>GeoMLAMA</t>
+          <t>DLAMA</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.68987372684939</v>
+        <v>0.7533247827402964</v>
       </c>
       <c r="C4" t="n">
-        <v>0.7393204622597835</v>
+        <v>0.7587982300872619</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>

</xml_diff>